<commit_message>
Update cost checks, overbilling and reports notebook
</commit_message>
<xml_diff>
--- a/reports/cost_check.xlsx
+++ b/reports/cost_check.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1415" uniqueCount="675">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1415" uniqueCount="676">
   <si>
     <t>CCS_Slip</t>
   </si>
@@ -1844,6 +1844,9 @@
   </si>
   <si>
     <t>0.9020</t>
+  </si>
+  <si>
+    <t>0.3410</t>
   </si>
   <si>
     <t>0.7140</t>
@@ -2704,13 +2707,13 @@
         <v>385</v>
       </c>
       <c r="AW2" t="s">
-        <v>616</v>
+        <v>617</v>
       </c>
       <c r="AX2" t="s">
-        <v>643</v>
+        <v>644</v>
       </c>
       <c r="AY2" t="s">
-        <v>674</v>
+        <v>675</v>
       </c>
     </row>
     <row r="3" spans="1:51">
@@ -2859,13 +2862,13 @@
         <v>386</v>
       </c>
       <c r="AW3" t="s">
-        <v>617</v>
+        <v>618</v>
       </c>
       <c r="AX3" t="s">
-        <v>644</v>
+        <v>645</v>
       </c>
       <c r="AY3" t="s">
-        <v>674</v>
+        <v>675</v>
       </c>
     </row>
     <row r="4" spans="1:51">
@@ -3017,10 +3020,10 @@
         <v>592</v>
       </c>
       <c r="AX4" t="s">
-        <v>645</v>
+        <v>646</v>
       </c>
       <c r="AY4" t="s">
-        <v>674</v>
+        <v>675</v>
       </c>
     </row>
     <row r="5" spans="1:51">
@@ -3169,13 +3172,13 @@
         <v>388</v>
       </c>
       <c r="AW5" t="s">
-        <v>618</v>
+        <v>619</v>
       </c>
       <c r="AX5" t="s">
-        <v>646</v>
+        <v>647</v>
       </c>
       <c r="AY5" t="s">
-        <v>674</v>
+        <v>675</v>
       </c>
     </row>
     <row r="6" spans="1:51">
@@ -3324,13 +3327,13 @@
         <v>389</v>
       </c>
       <c r="AW6" t="s">
-        <v>619</v>
+        <v>620</v>
       </c>
       <c r="AX6" t="s">
-        <v>647</v>
+        <v>648</v>
       </c>
       <c r="AY6" t="s">
-        <v>674</v>
+        <v>675</v>
       </c>
     </row>
     <row r="7" spans="1:51">
@@ -3479,13 +3482,13 @@
         <v>390</v>
       </c>
       <c r="AW7" t="s">
-        <v>620</v>
+        <v>621</v>
       </c>
       <c r="AX7" t="s">
-        <v>648</v>
+        <v>649</v>
       </c>
       <c r="AY7" t="s">
-        <v>674</v>
+        <v>675</v>
       </c>
     </row>
     <row r="8" spans="1:51">
@@ -3634,13 +3637,13 @@
         <v>391</v>
       </c>
       <c r="AW8" t="s">
-        <v>621</v>
+        <v>622</v>
       </c>
       <c r="AX8" t="s">
-        <v>649</v>
+        <v>650</v>
       </c>
       <c r="AY8" t="s">
-        <v>674</v>
+        <v>675</v>
       </c>
     </row>
     <row r="9" spans="1:51">
@@ -3789,13 +3792,13 @@
         <v>392</v>
       </c>
       <c r="AW9" t="s">
-        <v>622</v>
+        <v>623</v>
       </c>
       <c r="AX9" t="s">
-        <v>650</v>
+        <v>651</v>
       </c>
       <c r="AY9" t="s">
-        <v>674</v>
+        <v>675</v>
       </c>
     </row>
     <row r="10" spans="1:51">
@@ -3944,13 +3947,13 @@
         <v>393</v>
       </c>
       <c r="AW10" t="s">
-        <v>623</v>
+        <v>624</v>
       </c>
       <c r="AX10" t="s">
-        <v>651</v>
+        <v>652</v>
       </c>
       <c r="AY10" t="s">
-        <v>674</v>
+        <v>675</v>
       </c>
     </row>
     <row r="11" spans="1:51">
@@ -4099,13 +4102,13 @@
         <v>394</v>
       </c>
       <c r="AW11" t="s">
-        <v>624</v>
+        <v>625</v>
       </c>
       <c r="AX11" t="s">
-        <v>652</v>
+        <v>653</v>
       </c>
       <c r="AY11" t="s">
-        <v>674</v>
+        <v>675</v>
       </c>
     </row>
     <row r="12" spans="1:51">
@@ -4254,13 +4257,13 @@
         <v>384</v>
       </c>
       <c r="AW12" t="s">
-        <v>625</v>
+        <v>626</v>
       </c>
       <c r="AX12" t="s">
-        <v>653</v>
+        <v>654</v>
       </c>
       <c r="AY12" t="s">
-        <v>674</v>
+        <v>675</v>
       </c>
     </row>
     <row r="13" spans="1:51">
@@ -4409,13 +4412,13 @@
         <v>380</v>
       </c>
       <c r="AW13" t="s">
-        <v>626</v>
+        <v>627</v>
       </c>
       <c r="AX13" t="s">
-        <v>654</v>
+        <v>655</v>
       </c>
       <c r="AY13" t="s">
-        <v>674</v>
+        <v>675</v>
       </c>
     </row>
     <row r="14" spans="1:51">
@@ -4564,13 +4567,13 @@
         <v>388</v>
       </c>
       <c r="AW14" t="s">
-        <v>627</v>
+        <v>628</v>
       </c>
       <c r="AX14" t="s">
-        <v>655</v>
+        <v>656</v>
       </c>
       <c r="AY14" t="s">
-        <v>674</v>
+        <v>675</v>
       </c>
     </row>
     <row r="15" spans="1:51">
@@ -4719,13 +4722,13 @@
         <v>390</v>
       </c>
       <c r="AW15" t="s">
-        <v>628</v>
+        <v>629</v>
       </c>
       <c r="AX15" t="s">
-        <v>656</v>
+        <v>657</v>
       </c>
       <c r="AY15" t="s">
-        <v>674</v>
+        <v>675</v>
       </c>
     </row>
     <row r="16" spans="1:51">
@@ -4874,13 +4877,13 @@
         <v>395</v>
       </c>
       <c r="AW16" t="s">
-        <v>629</v>
+        <v>630</v>
       </c>
       <c r="AX16" t="s">
-        <v>657</v>
+        <v>658</v>
       </c>
       <c r="AY16" t="s">
-        <v>674</v>
+        <v>675</v>
       </c>
     </row>
     <row r="17" spans="1:51">
@@ -5029,13 +5032,13 @@
         <v>390</v>
       </c>
       <c r="AW17" t="s">
-        <v>630</v>
+        <v>631</v>
       </c>
       <c r="AX17" t="s">
-        <v>658</v>
+        <v>659</v>
       </c>
       <c r="AY17" t="s">
-        <v>674</v>
+        <v>675</v>
       </c>
     </row>
     <row r="18" spans="1:51">
@@ -5184,13 +5187,13 @@
         <v>396</v>
       </c>
       <c r="AW18" t="s">
-        <v>631</v>
+        <v>632</v>
       </c>
       <c r="AX18" t="s">
-        <v>659</v>
+        <v>660</v>
       </c>
       <c r="AY18" t="s">
-        <v>674</v>
+        <v>675</v>
       </c>
     </row>
     <row r="19" spans="1:51">
@@ -5339,13 +5342,13 @@
         <v>397</v>
       </c>
       <c r="AW19" t="s">
-        <v>632</v>
+        <v>633</v>
       </c>
       <c r="AX19" t="s">
-        <v>660</v>
+        <v>661</v>
       </c>
       <c r="AY19" t="s">
-        <v>674</v>
+        <v>675</v>
       </c>
     </row>
     <row r="20" spans="1:51">
@@ -5494,13 +5497,13 @@
         <v>391</v>
       </c>
       <c r="AW20" t="s">
-        <v>633</v>
+        <v>634</v>
       </c>
       <c r="AX20" t="s">
-        <v>661</v>
+        <v>662</v>
       </c>
       <c r="AY20" t="s">
-        <v>674</v>
+        <v>675</v>
       </c>
     </row>
     <row r="21" spans="1:51">
@@ -5652,10 +5655,10 @@
         <v>592</v>
       </c>
       <c r="AX21" t="s">
-        <v>662</v>
+        <v>663</v>
       </c>
       <c r="AY21" t="s">
-        <v>674</v>
+        <v>675</v>
       </c>
     </row>
     <row r="22" spans="1:51">
@@ -5804,13 +5807,13 @@
         <v>399</v>
       </c>
       <c r="AW22" t="s">
-        <v>634</v>
+        <v>635</v>
       </c>
       <c r="AX22" t="s">
-        <v>663</v>
+        <v>664</v>
       </c>
       <c r="AY22" t="s">
-        <v>674</v>
+        <v>675</v>
       </c>
     </row>
     <row r="23" spans="1:51">
@@ -5959,13 +5962,13 @@
         <v>397</v>
       </c>
       <c r="AW23" t="s">
-        <v>635</v>
+        <v>636</v>
       </c>
       <c r="AX23" t="s">
-        <v>664</v>
+        <v>665</v>
       </c>
       <c r="AY23" t="s">
-        <v>674</v>
+        <v>675</v>
       </c>
     </row>
     <row r="24" spans="1:51">
@@ -6087,13 +6090,13 @@
         <v>1</v>
       </c>
       <c r="AN24">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="AO24">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="AP24">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AQ24">
         <v>1</v>
@@ -6108,7 +6111,7 @@
         <v>598</v>
       </c>
       <c r="AU24" t="s">
-        <v>598</v>
+        <v>610</v>
       </c>
       <c r="AV24" t="s">
         <v>400</v>
@@ -6117,10 +6120,10 @@
         <v>592</v>
       </c>
       <c r="AX24" t="s">
-        <v>665</v>
+        <v>666</v>
       </c>
       <c r="AY24" t="s">
-        <v>674</v>
+        <v>675</v>
       </c>
     </row>
     <row r="25" spans="1:51">
@@ -6263,19 +6266,19 @@
         <v>598</v>
       </c>
       <c r="AU25" t="s">
-        <v>610</v>
+        <v>611</v>
       </c>
       <c r="AV25" t="s">
         <v>401</v>
       </c>
       <c r="AW25" t="s">
-        <v>636</v>
+        <v>637</v>
       </c>
       <c r="AX25" t="s">
-        <v>666</v>
+        <v>667</v>
       </c>
       <c r="AY25" t="s">
-        <v>674</v>
+        <v>675</v>
       </c>
     </row>
     <row r="26" spans="1:51">
@@ -6418,19 +6421,19 @@
         <v>598</v>
       </c>
       <c r="AU26" t="s">
-        <v>611</v>
+        <v>612</v>
       </c>
       <c r="AV26" t="s">
         <v>402</v>
       </c>
       <c r="AW26" t="s">
-        <v>637</v>
+        <v>638</v>
       </c>
       <c r="AX26" t="s">
-        <v>667</v>
+        <v>668</v>
       </c>
       <c r="AY26" t="s">
-        <v>674</v>
+        <v>675</v>
       </c>
     </row>
     <row r="27" spans="1:51">
@@ -6582,10 +6585,10 @@
         <v>592</v>
       </c>
       <c r="AX27" t="s">
-        <v>668</v>
+        <v>669</v>
       </c>
       <c r="AY27" t="s">
-        <v>674</v>
+        <v>675</v>
       </c>
     </row>
     <row r="28" spans="1:51">
@@ -6734,13 +6737,13 @@
         <v>384</v>
       </c>
       <c r="AW28" t="s">
-        <v>638</v>
+        <v>639</v>
       </c>
       <c r="AX28" t="s">
-        <v>669</v>
+        <v>670</v>
       </c>
       <c r="AY28" t="s">
-        <v>674</v>
+        <v>675</v>
       </c>
     </row>
     <row r="29" spans="1:51">
@@ -6883,19 +6886,19 @@
         <v>598</v>
       </c>
       <c r="AU29" t="s">
-        <v>612</v>
+        <v>613</v>
       </c>
       <c r="AV29" t="s">
         <v>384</v>
       </c>
       <c r="AW29" t="s">
-        <v>639</v>
+        <v>640</v>
       </c>
       <c r="AX29" t="s">
-        <v>670</v>
+        <v>671</v>
       </c>
       <c r="AY29" t="s">
-        <v>674</v>
+        <v>675</v>
       </c>
     </row>
     <row r="30" spans="1:51">
@@ -7038,19 +7041,19 @@
         <v>598</v>
       </c>
       <c r="AU30" t="s">
-        <v>613</v>
+        <v>614</v>
       </c>
       <c r="AV30" t="s">
         <v>404</v>
       </c>
       <c r="AW30" t="s">
-        <v>640</v>
+        <v>641</v>
       </c>
       <c r="AX30" t="s">
-        <v>671</v>
+        <v>672</v>
       </c>
       <c r="AY30" t="s">
-        <v>674</v>
+        <v>675</v>
       </c>
     </row>
     <row r="31" spans="1:51">
@@ -7193,19 +7196,19 @@
         <v>598</v>
       </c>
       <c r="AU31" t="s">
-        <v>614</v>
+        <v>615</v>
       </c>
       <c r="AV31" t="s">
         <v>405</v>
       </c>
       <c r="AW31" t="s">
-        <v>641</v>
+        <v>642</v>
       </c>
       <c r="AX31" t="s">
-        <v>672</v>
+        <v>673</v>
       </c>
       <c r="AY31" t="s">
-        <v>674</v>
+        <v>675</v>
       </c>
     </row>
     <row r="32" spans="1:51">
@@ -7348,19 +7351,19 @@
         <v>598</v>
       </c>
       <c r="AU32" t="s">
-        <v>615</v>
+        <v>616</v>
       </c>
       <c r="AV32" t="s">
         <v>406</v>
       </c>
       <c r="AW32" t="s">
-        <v>642</v>
+        <v>643</v>
       </c>
       <c r="AX32" t="s">
-        <v>673</v>
+        <v>674</v>
       </c>
       <c r="AY32" t="s">
-        <v>674</v>
+        <v>675</v>
       </c>
     </row>
   </sheetData>

</xml_diff>